<commit_message>
updated capella tests to run in headless mode
</commit_message>
<xml_diff>
--- a/src/main/resources/FeatureFiles/CapellaFormTestCase_chrome.xlsx
+++ b/src/main/resources/FeatureFiles/CapellaFormTestCase_chrome.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,9 +47,6 @@
     <t>beforeEach</t>
   </si>
   <si>
-    <t>openBrowser</t>
-  </si>
-  <si>
     <t>Chrome</t>
   </si>
   <si>
@@ -186,6 +183,9 @@
   </si>
   <si>
     <t>TC006 : Verify capella form will all fields filled with valid input except Check boxes</t>
+  </si>
+  <si>
+    <t>openHeadlessBrowser</t>
   </si>
 </sst>
 </file>
@@ -581,7 +581,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -599,7 +599,7 @@
     <col min="5" max="16384" width="8.75" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14.5">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -613,841 +613,841 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="14.5">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:4">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="14.5">
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="14.5">
-      <c r="B4" s="2" t="s">
+    <row r="5" spans="1:4">
+      <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="14.5">
-      <c r="B5" s="2" t="s">
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" ht="14.5">
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="14.5">
-      <c r="A7" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="B7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="D7" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="14.5">
-      <c r="B8" s="2" t="s">
+      <c r="D9" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="B10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="B11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="B13" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="B14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="B15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="B16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="B17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="B18" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="B19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="B21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="B22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="B23" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="B24" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="B25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="B26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="B27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="B28" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="B29" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="B30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="B31" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="B32" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="B33" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="14.5">
-      <c r="B9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="14.5">
-      <c r="B10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="14.5">
-      <c r="B11" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="14.5">
-      <c r="B12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="14.5">
-      <c r="B13" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="14.5">
-      <c r="B14" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="14.5">
-      <c r="B15" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="14.5">
-      <c r="B16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="14.5">
-      <c r="B17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="14.5">
-      <c r="B18" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="14.5">
-      <c r="B19" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="14.5">
-      <c r="A20" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="14.5">
-      <c r="B21" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="14.5">
-      <c r="B22" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="14.5">
-      <c r="B23" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="14.5">
-      <c r="B24" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="14.5">
-      <c r="B25" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="14.5">
-      <c r="B26" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="14.5">
-      <c r="B27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="14.5">
-      <c r="B28" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="14.5">
-      <c r="B29" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="14.5">
-      <c r="B30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="14.5">
-      <c r="B31" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="14.5">
-      <c r="B32" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="14.5">
-      <c r="B33" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="14.5">
-      <c r="A34" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="B35" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="B36" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="B37" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="B38" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4">
       <c r="B39" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="B40" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="B41" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="B42" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="B43" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="B44" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="B45" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="B46" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="B47" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B48" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C48" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="D48" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="B49" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="B50" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D50" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="B51" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C51" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="B52" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="B53" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="B54" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="B55" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C55" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="B56" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C56" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="B57" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="B58" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="B59" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B60" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="D60" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="B61" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="B62" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C62" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D62" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="B63" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C63" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D63" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="B64" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="B65" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="B66" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="B67" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="B68" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="B69" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="B70" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C70" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="B71" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C71" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="B72" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="B73" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B74" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C74" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="D74" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="B75" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="B76" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C76" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D76" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="B77" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C77" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D77" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="78" spans="1:4">
       <c r="B78" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="B79" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="B80" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D80" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="B81" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="B82" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="B83" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>